<commit_message>
Folha v3: coluna PRONTA passa a ser o turno que finalizou a peça (1, 2 ou 3)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019Px7p5mhzWYWbE6aV5W89g
</commit_message>
<xml_diff>
--- a/docs/folha-modelo/diario-de-bordo-v3.xlsx
+++ b/docs/folha-modelo/diario-de-bordo-v3.xlsx
@@ -633,9 +633,9 @@
     <col width="7" customWidth="1" min="14" max="14"/>
     <col width="6.6" customWidth="1" min="15" max="15"/>
     <col width="6.6" customWidth="1" min="16" max="16"/>
-    <col width="7.5" customWidth="1" min="17" max="17"/>
+    <col width="9.5" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="21" customWidth="1" min="19" max="19"/>
+    <col width="19" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -838,8 +838,9 @@
       <c r="P5" s="2" t="n"/>
       <c r="Q5" s="11" t="inlineStr">
         <is>
-          <t>PEÇA
-PRONTA ✓</t>
+          <t>PRONTA:
+TURNO QUE
+FINALIZOU</t>
         </is>
       </c>
       <c r="R5" s="11" t="inlineStr">
@@ -854,7 +855,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="n"/>
       <c r="B6" s="2" t="n"/>
       <c r="C6" s="2" t="n"/>
@@ -1701,7 +1702,7 @@
               <color rgb="FF111111"/>
               <sz val="8.5"/>
             </rPr>
-            <t xml:space="preserve">6. Marque </t>
+            <t xml:space="preserve">6. </t>
           </r>
           <r>
             <rPr>
@@ -1710,15 +1711,49 @@
               <color rgb="FF111111"/>
               <sz val="8.5"/>
             </rPr>
-            <t>✓ PRONTA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve"> quando a peça terminar. Não terminou? Deixe em branco e continue na próxima folha.
+            <t>Peça pronta?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF111111"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve"> Escreva em </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FF111111"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t>PRONTA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF111111"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve"> o </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FF111111"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t>turno que finalizou</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF111111"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve"> (1, 2 ou 3). Não terminou? Deixe em branco e continue na próxima folha.
 </t>
           </r>
           <r>
@@ -1778,7 +1813,7 @@
               <color rgb="FF111111"/>
               <sz val="8.5"/>
             </rPr>
-            <t xml:space="preserve"> o número da linha de cima. ✓ só na última linha.</t>
+            <t xml:space="preserve"> o número da linha de cima. O turno em PRONTA vai só na última linha.</t>
           </r>
         </is>
       </c>
@@ -2012,7 +2047,7 @@
               <color rgb="FF111111"/>
               <sz val="8.5"/>
             </rPr>
-            <t xml:space="preserve">VIGA · D51 · Trecho 1: 13:00–14:30 · Trecho 2: 15:30–17:00 · ✓
+            <t xml:space="preserve">VIGA · D51 · Trecho 1: 13:00–14:30 · Trecho 2: 15:30–17:00 · Pronta: 1
 </t>
           </r>
           <r>
@@ -2320,9 +2355,9 @@
     <col width="7" customWidth="1" min="14" max="14"/>
     <col width="6.6" customWidth="1" min="15" max="15"/>
     <col width="6.6" customWidth="1" min="16" max="16"/>
-    <col width="7.5" customWidth="1" min="17" max="17"/>
+    <col width="9.5" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="21" customWidth="1" min="19" max="19"/>
+    <col width="19" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -2480,8 +2515,9 @@
       <c r="P4" s="2" t="n"/>
       <c r="Q4" s="11" t="inlineStr">
         <is>
-          <t>PEÇA
-PRONTA ✓</t>
+          <t>PRONTA:
+TURNO QUE
+FINALIZOU</t>
         </is>
       </c>
       <c r="R4" s="11" t="inlineStr">
@@ -2496,7 +2532,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="2" t="n"/>
       <c r="B5" s="2" t="n"/>
       <c r="C5" s="2" t="n"/>
@@ -3256,7 +3292,7 @@
       <c r="G34" s="2" t="n"/>
       <c r="H34" s="23" t="inlineStr">
         <is>
-          <t>Peças prontas (nº de ✓)</t>
+          <t>Peças prontas (turno em PRONTA)</t>
         </is>
       </c>
       <c r="I34" s="2" t="n"/>
@@ -3317,7 +3353,24 @@
               <color rgb="FF111111"/>
               <sz val="8.5"/>
             </rPr>
-            <t>. ✓ quando a peça ficar pronta.</t>
+            <t xml:space="preserve">. Peça pronta: o </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FF111111"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t>turno que finalizou</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF111111"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve"> em PRONTA.</t>
           </r>
         </is>
       </c>
@@ -3517,9 +3570,9 @@
     <col width="7" customWidth="1" min="14" max="14"/>
     <col width="6.6" customWidth="1" min="15" max="15"/>
     <col width="6.6" customWidth="1" min="16" max="16"/>
-    <col width="7.5" customWidth="1" min="17" max="17"/>
+    <col width="9.5" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="21" customWidth="1" min="19" max="19"/>
+    <col width="19" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -3730,8 +3783,9 @@
       <c r="P5" s="2" t="n"/>
       <c r="Q5" s="11" t="inlineStr">
         <is>
-          <t>PEÇA
-PRONTA ✓</t>
+          <t>PRONTA:
+TURNO QUE
+FINALIZOU</t>
         </is>
       </c>
       <c r="R5" s="11" t="inlineStr">
@@ -3746,7 +3800,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
+    <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="n"/>
       <c r="B6" s="2" t="n"/>
       <c r="C6" s="2" t="n"/>
@@ -3854,10 +3908,8 @@
       <c r="N7" s="16" t="n"/>
       <c r="O7" s="17" t="n"/>
       <c r="P7" s="17" t="n"/>
-      <c r="Q7" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
+      <c r="Q7" s="18" t="n">
+        <v>1</v>
       </c>
       <c r="R7" s="7" t="n"/>
       <c r="S7" s="19" t="n"/>
@@ -3909,10 +3961,8 @@
       <c r="N8" s="16" t="n"/>
       <c r="O8" s="17" t="n"/>
       <c r="P8" s="17" t="n"/>
-      <c r="Q8" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
+      <c r="Q8" s="18" t="n">
+        <v>1</v>
       </c>
       <c r="R8" s="7" t="n"/>
       <c r="S8" s="19" t="n"/>
@@ -3956,10 +4006,8 @@
       <c r="N9" s="16" t="n"/>
       <c r="O9" s="17" t="n"/>
       <c r="P9" s="17" t="n"/>
-      <c r="Q9" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
+      <c r="Q9" s="18" t="n">
+        <v>1</v>
       </c>
       <c r="R9" s="7" t="n"/>
       <c r="S9" s="19" t="n"/>
@@ -4011,10 +4059,8 @@
       <c r="N10" s="16" t="n"/>
       <c r="O10" s="17" t="n"/>
       <c r="P10" s="17" t="n"/>
-      <c r="Q10" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
+      <c r="Q10" s="18" t="n">
+        <v>2</v>
       </c>
       <c r="R10" s="7" t="n"/>
       <c r="S10" s="19" t="inlineStr">
@@ -4133,10 +4179,8 @@
       <c r="N12" s="16" t="n"/>
       <c r="O12" s="17" t="n"/>
       <c r="P12" s="17" t="n"/>
-      <c r="Q12" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
+      <c r="Q12" s="18" t="n">
+        <v>2</v>
       </c>
       <c r="R12" s="7" t="n">
         <v>5</v>
@@ -4186,10 +4230,8 @@
       <c r="N13" s="16" t="n"/>
       <c r="O13" s="17" t="n"/>
       <c r="P13" s="17" t="n"/>
-      <c r="Q13" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
+      <c r="Q13" s="18" t="n">
+        <v>2</v>
       </c>
       <c r="R13" s="7" t="n"/>
       <c r="S13" s="19" t="n"/>
@@ -4233,10 +4275,8 @@
       <c r="N14" s="16" t="n"/>
       <c r="O14" s="17" t="n"/>
       <c r="P14" s="17" t="n"/>
-      <c r="Q14" s="18" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
+      <c r="Q14" s="18" t="n">
+        <v>3</v>
       </c>
       <c r="R14" s="7" t="n"/>
       <c r="S14" s="19" t="n"/>
@@ -5099,7 +5139,7 @@
               <color rgb="FF111111"/>
               <sz val="8.5"/>
             </rPr>
-            <t xml:space="preserve">6. Marque </t>
+            <t xml:space="preserve">6. </t>
           </r>
           <r>
             <rPr>
@@ -5108,15 +5148,49 @@
               <color rgb="FF111111"/>
               <sz val="8.5"/>
             </rPr>
-            <t>✓ PRONTA</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="FF111111"/>
-              <sz val="8.5"/>
-            </rPr>
-            <t xml:space="preserve"> quando a peça terminar. Não terminou? Deixe em branco e continue na próxima folha.
+            <t>Peça pronta?</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF111111"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve"> Escreva em </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FF111111"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t>PRONTA</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF111111"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve"> o </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FF111111"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t>turno que finalizou</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF111111"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve"> (1, 2 ou 3). Não terminou? Deixe em branco e continue na próxima folha.
 </t>
           </r>
           <r>
@@ -5176,7 +5250,7 @@
               <color rgb="FF111111"/>
               <sz val="8.5"/>
             </rPr>
-            <t xml:space="preserve"> o número da linha de cima. ✓ só na última linha.</t>
+            <t xml:space="preserve"> o número da linha de cima. O turno em PRONTA vai só na última linha.</t>
           </r>
         </is>
       </c>
@@ -5410,7 +5484,7 @@
               <color rgb="FF111111"/>
               <sz val="8.5"/>
             </rPr>
-            <t xml:space="preserve">VIGA · D51 · Trecho 1: 13:00–14:30 · Trecho 2: 15:30–17:00 · ✓
+            <t xml:space="preserve">VIGA · D51 · Trecho 1: 13:00–14:30 · Trecho 2: 15:30–17:00 · Pronta: 1
 </t>
           </r>
           <r>
@@ -5718,9 +5792,9 @@
     <col width="7" customWidth="1" min="14" max="14"/>
     <col width="6.6" customWidth="1" min="15" max="15"/>
     <col width="6.6" customWidth="1" min="16" max="16"/>
-    <col width="7.5" customWidth="1" min="17" max="17"/>
+    <col width="9.5" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="21" customWidth="1" min="19" max="19"/>
+    <col width="19" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -5890,8 +5964,9 @@
       <c r="P4" s="2" t="n"/>
       <c r="Q4" s="11" t="inlineStr">
         <is>
-          <t>PEÇA
-PRONTA ✓</t>
+          <t>PRONTA:
+TURNO QUE
+FINALIZOU</t>
         </is>
       </c>
       <c r="R4" s="11" t="inlineStr">
@@ -5906,7 +5981,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="2" t="n"/>
       <c r="B5" s="2" t="n"/>
       <c r="C5" s="2" t="n"/>
@@ -6666,7 +6741,7 @@
       <c r="G34" s="2" t="n"/>
       <c r="H34" s="23" t="inlineStr">
         <is>
-          <t>Peças prontas (nº de ✓)</t>
+          <t>Peças prontas (turno em PRONTA)</t>
         </is>
       </c>
       <c r="I34" s="2" t="n"/>
@@ -6727,7 +6802,24 @@
               <color rgb="FF111111"/>
               <sz val="8.5"/>
             </rPr>
-            <t>. ✓ quando a peça ficar pronta.</t>
+            <t xml:space="preserve">. Peça pronta: o </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <b val="1"/>
+              <color rgb="FF111111"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t>turno que finalizou</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="FF111111"/>
+              <sz val="8.5"/>
+            </rPr>
+            <t xml:space="preserve"> em PRONTA.</t>
           </r>
         </is>
       </c>

</xml_diff>